<commit_message>
Edited 3D Printing Files
Separated all 3D prints into their own separate files for users to configure on their build plate as desired.

Removed discrepancies from the print quantities and the updated list is now Full List of 3D Prints.xlsx.
</commit_message>
<xml_diff>
--- a/3D Printing Files/Full List of 3D Prints.xlsx
+++ b/3D Printing Files/Full List of 3D Prints.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveutk.sharepoint.com/sites/UT_DesktopMillingMachine/Shared Documents/General/GitHub-LC_CNC/LC-CNC/3D Printing Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveutk.sharepoint.com/sites/UT_DesktopMillingMachine/Shared Documents/General/GitHub-Landon/LC-CNC/3D Printing Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{1F10B019-920F-4413-835F-97FFA0B32539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C9F761F-9860-4506-BCEF-7F15CAC72ED5}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="8_{1F10B019-920F-4413-835F-97FFA0B32539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98EA1E1E-0499-45F8-B26A-9FD35C8EC188}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{4DF4BF29-A51F-4D9D-B524-88D1450504D2}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{4DF4BF29-A51F-4D9D-B524-88D1450504D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
   <si>
     <t>Enclosure</t>
   </si>
   <si>
-    <t>Name:</t>
-  </si>
-  <si>
     <t>Quantity:</t>
   </si>
   <si>
@@ -128,15 +125,6 @@
     <t>SmallJig</t>
   </si>
   <si>
-    <t>PSU Side Mount 3</t>
-  </si>
-  <si>
-    <t>big plate v4</t>
-  </si>
-  <si>
-    <t>small plate v4</t>
-  </si>
-  <si>
     <t>MagJackPlate</t>
   </si>
   <si>
@@ -146,23 +134,60 @@
     <t>FanGrills</t>
   </si>
   <si>
-    <t>Maybe?</t>
-  </si>
-  <si>
-    <t>Up to date?</t>
-  </si>
-  <si>
     <t>Connector cover top</t>
   </si>
   <si>
     <t>Connector cover bottom</t>
+  </si>
+  <si>
+    <t>3D printed files and quantities</t>
+  </si>
+  <si>
+    <t>Number of Machines:</t>
+  </si>
+  <si>
+    <t>File Name:</t>
+  </si>
+  <si>
+    <t>Probe touch plate</t>
+  </si>
+  <si>
+    <t>Collet Fan</t>
+  </si>
+  <si>
+    <t>DoveTailPlateFINAL.STEP</t>
+  </si>
+  <si>
+    <t>SmallPlateDoveTail.STEP</t>
+  </si>
+  <si>
+    <t>3PinDoveTailBracket025TEST.STEP</t>
+  </si>
+  <si>
+    <t>SingleDoveTail.STEP</t>
+  </si>
+  <si>
+    <t>5PinDoveTailBracket025TEST.STEP</t>
+  </si>
+  <si>
+    <t>PSU Side Mount 1 wCutout.STEP</t>
+  </si>
+  <si>
+    <t>OptoMount3.0.STEP</t>
+  </si>
+  <si>
+    <t>ContactorGuide.STEP</t>
+  </si>
+  <si>
+    <t>Drill and Box Prep Guides 
+(IF BOX IS NOT PREPARED FOR YOU)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,16 +203,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -195,13 +234,67 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,315 +629,399 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34CAE0CD-5F38-40D6-87CA-F68EF5A945FE}">
-  <dimension ref="A1:C40"/>
+  <dimension ref="B1:C52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.28515625" customWidth="1"/>
+    <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C4" s="5"/>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C6" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C7" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C8" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C9" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="C10" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C11" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
+      <c r="C12" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="5"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B32" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B10">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C34" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" s="5"/>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B11">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C38" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B40" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B41" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C42" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B43" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C43" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B45" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B46" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B47" s="6"/>
+      <c r="C47" s="6"/>
+    </row>
+    <row r="48" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B48" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48" s="5"/>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="6" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>1</v>
-      </c>
-      <c r="B32" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="C49" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="C50" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>33</v>
-      </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>34</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
-        <v>35</v>
+      <c r="C51" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B52" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C52" s="6">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -854,26 +1031,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="fb0bfce0-b493-4733-b695-336371de64d4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a816e368-bd7d-4e73-ae60-f7bbf4d187c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010049C730614A98FF4D948BAAFAA2763638" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="71752533c218a459f0bd7314a8d27046">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a816e368-bd7d-4e73-ae60-f7bbf4d187c7" xmlns:ns3="fb0bfce0-b493-4733-b695-336371de64d4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="56df45e61c8cd6f396207a6803100ce0" ns2:_="" ns3:_="">
     <xsd:import namespace="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
@@ -1086,26 +1243,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12287FA2-93E6-4971-BE9B-FA34AA5244CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fb0bfce0-b493-4733-b695-336371de64d4"/>
-    <ds:schemaRef ds:uri="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F07644A4-9A62-4B7D-AF73-0355BCF7E4A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="fb0bfce0-b493-4733-b695-336371de64d4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a816e368-bd7d-4e73-ae60-f7bbf4d187c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B2CF0CF-210A-4906-8EBD-77C2149273B7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1122,4 +1280,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F07644A4-9A62-4B7D-AF73-0355BCF7E4A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12287FA2-93E6-4971-BE9B-FA34AA5244CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fb0bfce0-b493-4733-b695-336371de64d4"/>
+    <ds:schemaRef ds:uri="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated PSU Mount and Optocoupler Mount 3D Prints
PSU Side Mount 1 w/ cutout -> PSU Side Mount 3. This new print addresses issues with the mounting to the electrical grid.

OptoMount3.0 -> OptoMount5.0. This model includes the single channel optocoupler onto the 4 channel optocoupler mount.

The Full List of 3D Prints have been updated to reflect these changes.
</commit_message>
<xml_diff>
--- a/3D Printing Files/Full List of 3D Prints.xlsx
+++ b/3D Printing Files/Full List of 3D Prints.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveutk.sharepoint.com/sites/UT_DesktopMillingMachine/Shared Documents/General/GitHub-Landon/LC-CNC/3D Printing Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{1F10B019-920F-4413-835F-97FFA0B32539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98EA1E1E-0499-45F8-B26A-9FD35C8EC188}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="8_{1F10B019-920F-4413-835F-97FFA0B32539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9EC5FD4-9AFB-49F9-AE4B-D877242ADE23}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{4DF4BF29-A51F-4D9D-B524-88D1450504D2}"/>
   </bookViews>
@@ -155,32 +155,32 @@
     <t>Collet Fan</t>
   </si>
   <si>
-    <t>DoveTailPlateFINAL.STEP</t>
-  </si>
-  <si>
-    <t>SmallPlateDoveTail.STEP</t>
-  </si>
-  <si>
-    <t>3PinDoveTailBracket025TEST.STEP</t>
-  </si>
-  <si>
-    <t>SingleDoveTail.STEP</t>
-  </si>
-  <si>
-    <t>5PinDoveTailBracket025TEST.STEP</t>
-  </si>
-  <si>
-    <t>PSU Side Mount 1 wCutout.STEP</t>
-  </si>
-  <si>
-    <t>OptoMount3.0.STEP</t>
-  </si>
-  <si>
-    <t>ContactorGuide.STEP</t>
-  </si>
-  <si>
     <t>Drill and Box Prep Guides 
 (IF BOX IS NOT PREPARED FOR YOU)</t>
+  </si>
+  <si>
+    <t>DoveTailPlateFINAL</t>
+  </si>
+  <si>
+    <t>SmallPlateDoveTail</t>
+  </si>
+  <si>
+    <t>3PinDoveTailBracket025TEST</t>
+  </si>
+  <si>
+    <t>SingleDoveTail</t>
+  </si>
+  <si>
+    <t>5PinDoveTailBracket025TEST</t>
+  </si>
+  <si>
+    <t>OptoMount5.0</t>
+  </si>
+  <si>
+    <t>ContactorGuide</t>
+  </si>
+  <si>
+    <t>PSU Side Mount 3</t>
   </si>
 </sst>
 </file>
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -291,7 +291,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -310,6 +309,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -877,7 +880,7 @@
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C33" s="6">
@@ -885,7 +888,7 @@
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C34" s="6">
@@ -911,40 +914,40 @@
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B38" s="7" t="s">
-        <v>38</v>
+      <c r="B38" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="C38" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B39" s="7" t="s">
-        <v>39</v>
+      <c r="B39" s="6" t="s">
+        <v>40</v>
       </c>
       <c r="C39" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B40" s="7" t="s">
-        <v>40</v>
+      <c r="B40" s="6" t="s">
+        <v>41</v>
       </c>
       <c r="C40" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="7" t="s">
-        <v>41</v>
+      <c r="B41" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="C41" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B42" s="7" t="s">
-        <v>42</v>
+      <c r="B42" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="C42" s="6">
         <v>1</v>
@@ -959,15 +962,15 @@
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B44" s="7" t="s">
-        <v>43</v>
+      <c r="B44" s="6" t="s">
+        <v>46</v>
       </c>
       <c r="C44" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="6" t="s">
         <v>44</v>
       </c>
       <c r="C45" s="6">
@@ -987,8 +990,8 @@
       <c r="C47" s="6"/>
     </row>
     <row r="48" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B48" s="8" t="s">
-        <v>46</v>
+      <c r="B48" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="C48" s="5"/>
     </row>
@@ -1017,7 +1020,7 @@
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B52" s="7" t="s">
+      <c r="B52" s="6" t="s">
         <v>45</v>
       </c>
       <c r="C52" s="6">
@@ -1031,6 +1034,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="fb0bfce0-b493-4733-b695-336371de64d4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a816e368-bd7d-4e73-ae60-f7bbf4d187c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010049C730614A98FF4D948BAAFAA2763638" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="71752533c218a459f0bd7314a8d27046">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a816e368-bd7d-4e73-ae60-f7bbf4d187c7" xmlns:ns3="fb0bfce0-b493-4733-b695-336371de64d4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="56df45e61c8cd6f396207a6803100ce0" ns2:_="" ns3:_="">
     <xsd:import namespace="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
@@ -1243,27 +1266,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12287FA2-93E6-4971-BE9B-FA34AA5244CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fb0bfce0-b493-4733-b695-336371de64d4"/>
+    <ds:schemaRef ds:uri="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="fb0bfce0-b493-4733-b695-336371de64d4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a816e368-bd7d-4e73-ae60-f7bbf4d187c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F07644A4-9A62-4B7D-AF73-0355BCF7E4A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B2CF0CF-210A-4906-8EBD-77C2149273B7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1280,23 +1302,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F07644A4-9A62-4B7D-AF73-0355BCF7E4A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12287FA2-93E6-4971-BE9B-FA34AA5244CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fb0bfce0-b493-4733-b695-336371de64d4"/>
-    <ds:schemaRef ds:uri="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>